<commit_message>
hopefully fixed notebooks, and cleanup
</commit_message>
<xml_diff>
--- a/Versionen/aug-14/game_data.xlsx
+++ b/Versionen/aug-14/game_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Documents\_Privat\Coding\KlimSta\Versionen\aug-14\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schneids\code\KlimSta-Brettspiel\Versionen\aug-14\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63A1FADE-E50F-4C6C-B5E5-1111E92B6F82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="873" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-18060" yWindow="-17388" windowWidth="30936" windowHeight="16776" tabRatio="873" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Massnahmenkarten Spielwerte" sheetId="1" r:id="rId1"/>
@@ -73,9 +73,9 @@
   <commentList>
     <comment ref="C1" authorId="0" shapeId="0" xr:uid="{884F3275-8B47-4A24-9A63-26455AFB7D59}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Kommentarthread]
+Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
+Kommentar:
     KgCO2/m²a</t>
       </text>
     </comment>
@@ -92,18 +92,18 @@
   <commentList>
     <comment ref="C2" authorId="0" shapeId="0" xr:uid="{EF592111-A8C2-4853-9B03-5FD652A65E13}">
       <text>
-        <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t xml:space="preserve">[Kommentarthread]
+Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
+Kommentar:
     €/m²
 </t>
       </text>
     </comment>
     <comment ref="H2" authorId="1" shapeId="0" xr:uid="{42E090DF-C6E0-4ACF-94D0-539FD66BF793}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Kommentarthread]
+Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
+Kommentar:
     Geld token</t>
       </text>
     </comment>
@@ -2080,7 +2080,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="144">
+  <cellXfs count="143">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2489,41 +2489,14 @@
     <xf numFmtId="0" fontId="2" fillId="10" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="81">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Roboto"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF6D9EEB"/>
-          <bgColor rgb="FF6D9EEB"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="90" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2531,9 +2504,6 @@
           <bgColor rgb="FFB7E1CD"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -3092,6 +3062,33 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Roboto"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF6D9EEB"/>
+          <bgColor rgb="FF6D9EEB"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="90" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -3592,11 +3589,11 @@
     <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="REAL Stromspeicher"/>
     <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="REAL Wärmeschutz"/>
     <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="REAL Wärmepumpen-Effizienz"/>
-    <tableColumn id="28" xr3:uid="{B7683582-900D-4F40-82AF-9122419510A0}" name="Freitext" dataDxfId="0"/>
+    <tableColumn id="28" xr3:uid="{B7683582-900D-4F40-82AF-9122419510A0}" name="Freitext" dataDxfId="42"/>
     <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Voraussetzung Spalte"/>
     <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Voraussetzung Wert"/>
     <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Voraussetzung Wert NICHT"/>
-    <tableColumn id="26" xr3:uid="{FDB4847F-B10D-4845-B90B-E9D5F945F1B7}" name="EffektParsed" dataDxfId="42">
+    <tableColumn id="26" xr3:uid="{FDB4847F-B10D-4845-B90B-E9D5F945F1B7}" name="EffektParsed" dataDxfId="41">
       <calculatedColumnFormula>_xlfn.TEXTJOIN(
 "XX",
 TRUE,
@@ -3610,7 +3607,7 @@
 IF(D2="FW","XXFW",IF(D2="BIO","XXBI",IF(D2="ABWWP","XXWP",IF(D2="WP","XXWP",IF(D2="GG","XXGG","")))))
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="27" xr3:uid="{BE3C4938-8F19-4E3F-9C9A-34227C4C8923}" name="Beschreibung" dataDxfId="2">
+    <tableColumn id="27" xr3:uid="{BE3C4938-8F19-4E3F-9C9A-34227C4C8923}" name="Beschreibung" dataDxfId="40">
       <calculatedColumnFormula>CHAR(34)&amp;VLOOKUP(Table1[[#This Row],[Name]],'Massnahmenkarten Texte'!A:C,3,FALSE)&amp;CHAR(34)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3638,8 +3635,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table3" displayName="Table3" ref="A1:E34">
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Wert"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Real" dataDxfId="41"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Spiel" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Real" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Spiel" dataDxfId="38"/>
     <tableColumn id="5" xr3:uid="{16BD6806-29CB-4A81-B6F6-E74363828D03}" name="Skalierung real &gt; spiel"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Einheit"/>
   </tableColumns>
@@ -3672,19 +3669,19 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table6" displayName="Table6" ref="A1:L11">
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="WS"/>
-    <tableColumn id="12" xr3:uid="{EB8234D1-70DE-48AE-82B3-197397D4EA50}" name="HWB" dataDxfId="39"/>
-    <tableColumn id="7" xr3:uid="{382715DF-E649-4C68-8229-17F79CFD05E9}" name="Gas Real" dataDxfId="38"/>
-    <tableColumn id="8" xr3:uid="{9D3BFB1F-D194-4CFF-801A-646B03B69223}" name="Biomasse Real" dataDxfId="37"/>
-    <tableColumn id="9" xr3:uid="{92D64809-6003-4492-A647-B5959B9DDB64}" name="Fernwärme Real" dataDxfId="36"/>
-    <tableColumn id="10" xr3:uid="{08723E33-0A65-4BFC-9E7A-BA30B56D6C93}" name="Grünes Gas Real" dataDxfId="35"/>
-    <tableColumn id="11" xr3:uid="{308CC45B-DB70-43B9-B4BC-DFAA9033E01B}" name="Wärmepumpe Real" dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Gas" dataDxfId="33">
+    <tableColumn id="12" xr3:uid="{EB8234D1-70DE-48AE-82B3-197397D4EA50}" name="HWB" dataDxfId="37"/>
+    <tableColumn id="7" xr3:uid="{382715DF-E649-4C68-8229-17F79CFD05E9}" name="Gas Real" dataDxfId="36"/>
+    <tableColumn id="8" xr3:uid="{9D3BFB1F-D194-4CFF-801A-646B03B69223}" name="Biomasse Real" dataDxfId="35"/>
+    <tableColumn id="9" xr3:uid="{92D64809-6003-4492-A647-B5959B9DDB64}" name="Fernwärme Real" dataDxfId="34"/>
+    <tableColumn id="10" xr3:uid="{08723E33-0A65-4BFC-9E7A-BA30B56D6C93}" name="Grünes Gas Real" dataDxfId="33"/>
+    <tableColumn id="11" xr3:uid="{308CC45B-DB70-43B9-B4BC-DFAA9033E01B}" name="Wärmepumpe Real" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Gas" dataDxfId="31">
       <calculatedColumnFormula>Table6[[#This Row],[Gas Real]]*years_per_round</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Biomasse">
       <calculatedColumnFormula>Table6[[#This Row],[Biomasse Real]]*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Fernwärme" dataDxfId="32">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Fernwärme" dataDxfId="30">
       <calculatedColumnFormula>Table6[[#This Row],[Fernwärme Real]]*years_per_round</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="Grünes Gas">
@@ -3702,35 +3699,35 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Table6_2" displayName="Table6_2" ref="A1:L11">
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="WS"/>
-    <tableColumn id="12" xr3:uid="{0F5289D2-6D79-4CC0-B64B-353B2E52E442}" name="HWB" dataDxfId="31"/>
-    <tableColumn id="7" xr3:uid="{7EE7A865-A9C3-4293-93B4-6A7F6B0D0739}" name="Gas Real" dataDxfId="30">
+    <tableColumn id="12" xr3:uid="{0F5289D2-6D79-4CC0-B64B-353B2E52E442}" name="HWB" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{7EE7A865-A9C3-4293-93B4-6A7F6B0D0739}" name="Gas Real" dataDxfId="28">
       <calculatedColumnFormula>Table6_2[[#This Row],[HWB]]*'Mapping RealwerteSpielwerte'!$B$23</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{B9056603-4120-4751-8FD5-39C0A331CEB9}" name="Biomasse Real" dataDxfId="29">
+    <tableColumn id="8" xr3:uid="{B9056603-4120-4751-8FD5-39C0A331CEB9}" name="Biomasse Real" dataDxfId="27">
       <calculatedColumnFormula>Table6_2[[#This Row],[HWB]]*'Mapping RealwerteSpielwerte'!$B$24</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{775B0FD7-CE79-4EF3-8952-C905936C6A82}" name="Fernwärme Real" dataDxfId="28">
+    <tableColumn id="9" xr3:uid="{775B0FD7-CE79-4EF3-8952-C905936C6A82}" name="Fernwärme Real" dataDxfId="26">
       <calculatedColumnFormula>Table6_2[[#This Row],[HWB]]*'Mapping RealwerteSpielwerte'!$B$25</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{600AB853-60A0-47F9-B6B9-14F74CC0E0AE}" name="Grünes Gas Real" dataDxfId="27">
+    <tableColumn id="10" xr3:uid="{600AB853-60A0-47F9-B6B9-14F74CC0E0AE}" name="Grünes Gas Real" dataDxfId="25">
       <calculatedColumnFormula>Table6_2[[#This Row],[HWB]]*'Mapping RealwerteSpielwerte'!$B$26</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{1611B9F2-405C-4348-B6D7-02BE82C080AD}" name="Wärmepumpe Real" dataDxfId="26">
+    <tableColumn id="11" xr3:uid="{1611B9F2-405C-4348-B6D7-02BE82C080AD}" name="Wärmepumpe Real" dataDxfId="24">
       <calculatedColumnFormula>0</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Gas" dataDxfId="25">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Gas" dataDxfId="23">
       <calculatedColumnFormula>-Table6_2[[#This Row],[Gas Real]]*'Mapping RealwerteSpielwerte'!$C$23+heizkosten_baseline</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Biomasse" dataDxfId="24">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Biomasse" dataDxfId="22">
       <calculatedColumnFormula>-Table6_2[[#This Row],[Biomasse Real]]*'Mapping RealwerteSpielwerte'!$C$24+heizkosten_baseline</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Fernwärme" dataDxfId="23">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Fernwärme" dataDxfId="21">
       <calculatedColumnFormula>-Table6_2[[#This Row],[Fernwärme Real]]*'Mapping RealwerteSpielwerte'!$C$25+heizkosten_baseline</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="Grünes Gas" dataDxfId="22">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="Grünes Gas" dataDxfId="20">
       <calculatedColumnFormula>-Table6_2[[#This Row],[Grünes Gas Real]]*'Mapping RealwerteSpielwerte'!$C$26+heizkosten_baseline</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="Wärmepumpe" dataDxfId="21">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="Wärmepumpe" dataDxfId="19">
       <calculatedColumnFormula>-Table6_2[[#This Row],[Wärmepumpe Real]]*'Mapping RealwerteSpielwerte'!$C$27+heizkosten_baseline</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3745,23 +3742,23 @@
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="WS"/>
-    <tableColumn id="8" xr3:uid="{9A60DCE1-E93F-4731-A39D-070BBC8CF024}" name="HWB" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{DB8D5F2F-7A4D-4517-BD90-EB468A9472F9}" name="Effizienz 0" dataDxfId="19">
+    <tableColumn id="8" xr3:uid="{9A60DCE1-E93F-4731-A39D-070BBC8CF024}" name="HWB" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{DB8D5F2F-7A4D-4517-BD90-EB468A9472F9}" name="Effizienz 0" dataDxfId="17">
       <calculatedColumnFormula>Table7[[#This Row],[HWB]]/real_zu_spiel_strombedarf/COP_0</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Effizienz 1" dataDxfId="18">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Effizienz 1" dataDxfId="16">
       <calculatedColumnFormula>Table7[[#This Row],[HWB]]/real_zu_spiel_strombedarf/COP_1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Effizienz 2" dataDxfId="17">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Effizienz 2" dataDxfId="15">
       <calculatedColumnFormula>Table7[[#This Row],[HWB]]/real_zu_spiel_strombedarf/COP_2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Effizienz 3" dataDxfId="16">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Effizienz 3" dataDxfId="14">
       <calculatedColumnFormula>Table7[[#This Row],[HWB]]/real_zu_spiel_strombedarf/COP_3</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="Effizienz 4" dataDxfId="15">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="Effizienz 4" dataDxfId="13">
       <calculatedColumnFormula>Table7[[#This Row],[HWB]]/real_zu_spiel_strombedarf/COP_4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="Effizienz 5" dataDxfId="14">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="Effizienz 5" dataDxfId="12">
       <calculatedColumnFormula>Table7[[#This Row],[HWB]]/real_zu_spiel_strombedarf/COP_5</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3773,37 +3770,37 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="Table8" displayName="Table8" ref="A1:L37">
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="Netzbezug"/>
-    <tableColumn id="7" xr3:uid="{FA3BADB2-767D-406F-AE0E-3FD85C94E47C}" name="Netzbezug Real" dataDxfId="13">
+    <tableColumn id="7" xr3:uid="{FA3BADB2-767D-406F-AE0E-3FD85C94E47C}" name="Netzbezug Real" dataDxfId="11">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug]]*real_zu_spiel_netzbezug</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{7CF654A3-746E-45BB-8FE8-D85A1A2F26B3}" name="Kosten Real" dataDxfId="12">
+    <tableColumn id="12" xr3:uid="{7CF654A3-746E-45BB-8FE8-D85A1A2F26B3}" name="Kosten Real" dataDxfId="10">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*'Mapping RealwerteSpielwerte'!$B$27</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Budget" dataDxfId="11">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Budget" dataDxfId="9">
       <calculatedColumnFormula>-Table8[[#This Row],[Kosten Real]]*'Mapping RealwerteSpielwerte'!$C$27</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{CF2B80D5-564A-4F28-96D5-E05D40FB1362}" name="Emissionen Runde 1 Real" dataDxfId="10">
+    <tableColumn id="8" xr3:uid="{CF2B80D5-564A-4F28-96D5-E05D40FB1362}" name="Emissionen Runde 1 Real" dataDxfId="8">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{DDA1FEAD-C691-4D07-9868-BA59E3083198}" name="Emissionen Runde 2 Real" dataDxfId="9">
+    <tableColumn id="9" xr3:uid="{DDA1FEAD-C691-4D07-9868-BA59E3083198}" name="Emissionen Runde 2 Real" dataDxfId="7">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{FA64A352-3640-4484-B5E7-A06D893CF066}" name="Emissionen Runde 3 Real" dataDxfId="8">
+    <tableColumn id="10" xr3:uid="{FA64A352-3640-4484-B5E7-A06D893CF066}" name="Emissionen Runde 3 Real" dataDxfId="6">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{D2D0C651-2DB4-4AE8-8AC2-5459168B14AC}" name="Emissionen Runde 4 Real" dataDxfId="7">
+    <tableColumn id="11" xr3:uid="{D2D0C651-2DB4-4AE8-8AC2-5459168B14AC}" name="Emissionen Runde 4 Real" dataDxfId="5">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="SP Runde 1" dataDxfId="6">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="SP Runde 1" dataDxfId="4">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="SP Runde 2" dataDxfId="5">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="SP Runde 2" dataDxfId="3">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="SP Runde 3" dataDxfId="4">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="SP Runde 3" dataDxfId="2">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="SP Runde 4" dataDxfId="3">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="SP Runde 4" dataDxfId="1">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4069,7 +4066,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:AB1003"/>
-  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.453125" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -4467,7 +4464,7 @@
       <c r="V6" s="22">
         <v>1</v>
       </c>
-      <c r="W6" s="143" t="s">
+      <c r="W6" s="85" t="s">
         <v>422</v>
       </c>
       <c r="X6" s="54" t="s">
@@ -4534,7 +4531,7 @@
       </c>
       <c r="U7" s="21"/>
       <c r="V7" s="39"/>
-      <c r="W7" s="143" t="s">
+      <c r="W7" s="85" t="s">
         <v>423</v>
       </c>
       <c r="X7" s="32" t="s">
@@ -4597,7 +4594,7 @@
       <c r="T8" s="51"/>
       <c r="U8" s="21"/>
       <c r="V8" s="39"/>
-      <c r="W8" s="143" t="s">
+      <c r="W8" s="85" t="s">
         <v>422</v>
       </c>
       <c r="X8" s="32" t="s">
@@ -4919,7 +4916,7 @@
       </c>
       <c r="U13" s="21"/>
       <c r="V13" s="39"/>
-      <c r="W13" s="143" t="s">
+      <c r="W13" s="85" t="s">
         <v>422</v>
       </c>
       <c r="X13" s="54" t="s">
@@ -5510,7 +5507,7 @@
       <c r="V22" s="22">
         <v>1</v>
       </c>
-      <c r="W22" s="143"/>
+      <c r="W22" s="85"/>
       <c r="X22" s="32"/>
       <c r="Y22" s="32"/>
       <c r="Z22" s="12"/>
@@ -5571,7 +5568,7 @@
       <c r="V23" s="22">
         <v>2</v>
       </c>
-      <c r="W23" s="143" t="s">
+      <c r="W23" s="85" t="s">
         <v>429</v>
       </c>
       <c r="X23" s="54" t="s">
@@ -5640,7 +5637,7 @@
       <c r="V24" s="22">
         <v>2</v>
       </c>
-      <c r="W24" s="143" t="s">
+      <c r="W24" s="85" t="s">
         <v>430</v>
       </c>
       <c r="X24" s="32" t="s">
@@ -5707,7 +5704,7 @@
       <c r="V25" s="22">
         <v>1</v>
       </c>
-      <c r="W25" s="143" t="s">
+      <c r="W25" s="85" t="s">
         <v>429</v>
       </c>
       <c r="X25" s="32" t="s">
@@ -5776,7 +5773,7 @@
       <c r="V26" s="22">
         <v>2</v>
       </c>
-      <c r="W26" s="143" t="s">
+      <c r="W26" s="85" t="s">
         <v>429</v>
       </c>
       <c r="X26" s="54" t="s">
@@ -5851,7 +5848,7 @@
       <c r="V27" s="22">
         <v>1</v>
       </c>
-      <c r="W27" s="143"/>
+      <c r="W27" s="85"/>
       <c r="X27" s="54"/>
       <c r="Y27" s="54"/>
       <c r="Z27" s="54"/>
@@ -5912,7 +5909,7 @@
       <c r="V28" s="22">
         <v>2</v>
       </c>
-      <c r="W28" s="143" t="s">
+      <c r="W28" s="85" t="s">
         <v>430</v>
       </c>
       <c r="X28" s="54" t="s">
@@ -8316,7 +8313,7 @@
       <c r="V67" s="22">
         <v>2</v>
       </c>
-      <c r="W67" s="143"/>
+      <c r="W67" s="85"/>
       <c r="X67" s="32"/>
       <c r="Y67" s="32"/>
       <c r="Z67" s="32"/>
@@ -8444,7 +8441,7 @@
       <c r="V69" s="22">
         <v>1</v>
       </c>
-      <c r="W69" s="143"/>
+      <c r="W69" s="85"/>
       <c r="X69" s="54"/>
       <c r="Y69" s="54"/>
       <c r="Z69" s="54"/>
@@ -8522,7 +8519,7 @@
       <c r="V70" s="22">
         <v>2</v>
       </c>
-      <c r="W70" s="143"/>
+      <c r="W70" s="85"/>
       <c r="X70" s="54"/>
       <c r="Y70" s="54"/>
       <c r="Z70" s="54"/>
@@ -8646,7 +8643,7 @@
       <c r="V72" s="22">
         <v>2</v>
       </c>
-      <c r="W72" s="143"/>
+      <c r="W72" s="85"/>
       <c r="X72" s="32"/>
       <c r="Y72" s="32"/>
       <c r="Z72" s="32"/>
@@ -8827,7 +8824,7 @@
       <c r="V75" s="78">
         <v>1</v>
       </c>
-      <c r="W75" s="143"/>
+      <c r="W75" s="85"/>
       <c r="X75" s="54"/>
       <c r="Y75" s="54"/>
       <c r="Z75" s="54"/>
@@ -33924,8 +33921,8 @@
       <c r="Y1003" s="32"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="O2:O103 O1:W1 Q76:W103">
-    <cfRule type="expression" dxfId="1" priority="1">
+  <conditionalFormatting sqref="O1:W1 O2:O103 Q76:W103">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>"T"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -33949,7 +33946,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:V996"/>
-  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.453125" customWidth="1"/>
     <col min="2" max="4" width="35.1796875" customWidth="1"/>
@@ -58701,7 +58698,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:M35"/>
-  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.54296875" customWidth="1"/>
     <col min="5" max="5" width="21.7265625" customWidth="1"/>
@@ -59270,7 +59267,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:M6"/>
-  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.54296875" customWidth="1"/>
     <col min="2" max="2" width="17.26953125" customWidth="1"/>
@@ -59538,7 +59535,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="9" max="9" width="12.81640625" customWidth="1"/>
     <col min="10" max="10" width="13.81640625" customWidth="1"/>
@@ -60035,7 +60032,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="9" max="9" width="12.81640625" customWidth="1"/>
     <col min="10" max="10" width="13.81640625" customWidth="1"/>
@@ -60606,7 +60603,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:H25"/>
-  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="8" width="13.1796875" customWidth="1"/>
   </cols>
@@ -61049,7 +61046,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:L37"/>
-  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.7265625" customWidth="1"/>
     <col min="10" max="13" width="14" customWidth="1"/>

</xml_diff>